<commit_message>
orderDetail : retour à 0..* et short déplacé au bon niveau 8ded7fffc56465e5e419acd48191c473801e9e27
</commit_message>
<xml_diff>
--- a/nr-doc-core-service-request/ig/StructureDefinition-fr-core-service-request.xlsx
+++ b/nr-doc-core-service-request/ig/StructureDefinition-fr-core-service-request.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1919" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1770" uniqueCount="453">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-23T09:36:51+00:00</t>
+    <t>2026-07-23T09:46:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -869,7 +869,7 @@
 </t>
   </si>
   <si>
-    <t>Additional order information</t>
+    <t>Résultat de la demande</t>
   </si>
   <si>
     <t>Additional details and instructions about the how the services are to be delivered.   For example, and order for a urinary catheter may have an order detail for an external or indwelling catheter, or an order for a bandage may require additional instructions specifying how the bandage should be applied.</t>
@@ -891,596 +891,514 @@
     <t>NTE</t>
   </si>
   <si>
-    <t>ServiceRequest.orderDetail.id</t>
+    <t>ServiceRequest.quantity[x]</t>
+  </si>
+  <si>
+    <t>Quantity
+RatioRange</t>
+  </si>
+  <si>
+    <t>Service amount</t>
+  </si>
+  <si>
+    <t>An amount of service being requested which can be a quantity ( for example $1,500 home modification), a ratio ( for example, 20 half day visits per month), or a range (2.0 to 1.8 Gy per fraction).</t>
+  </si>
+  <si>
+    <t>When ordering a service the number of service items may need to be specified separately from the the service item.</t>
+  </si>
+  <si>
+    <t>.quantity</t>
+  </si>
+  <si>
+    <t>ServiceRequest.subject</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(Patient|4.0.1|Group|4.0.1|Location|4.0.1|Device|4.0.1)
+</t>
+  </si>
+  <si>
+    <t>Individual or Entity the service is ordered for</t>
+  </si>
+  <si>
+    <t>On whom or what the service is to be performed. This is usually a human patient, but can also be requested on animals, groups of humans or animals, devices such as dialysis machines, or even locations (typically for environmental scans).</t>
+  </si>
+  <si>
+    <t>Request.subject</t>
+  </si>
+  <si>
+    <t>PID</t>
+  </si>
+  <si>
+    <t>.participation[typeCode=SBJ].role</t>
+  </si>
+  <si>
+    <t>FiveWs.subject</t>
+  </si>
+  <si>
+    <t>ClinicalStatement.subject</t>
+  </si>
+  <si>
+    <t>ServiceRequest.encounter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">context
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(Encounter|4.0.1)
+</t>
+  </si>
+  <si>
+    <t>Encounter in which the request was created</t>
+  </si>
+  <si>
+    <t>An encounter that provides additional information about the healthcare context in which this request is made.</t>
+  </si>
+  <si>
+    <t>Request.encounter</t>
+  </si>
+  <si>
+    <t>PV1</t>
+  </si>
+  <si>
+    <t>.inboundRelationship(typeCode=COMP].source[classCode&lt;=PCPR, moodCode=EVN]</t>
+  </si>
+  <si>
+    <t>FiveWs.context</t>
+  </si>
+  <si>
+    <t>ClinicalStatement.encounter</t>
+  </si>
+  <si>
+    <t>ServiceRequest.occurrence[x]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">schedule
+</t>
+  </si>
+  <si>
+    <t>dateTime
+PeriodTiming</t>
+  </si>
+  <si>
+    <t>Date prévisionnelle de l'examen, du suivi, de l'objectif</t>
+  </si>
+  <si>
+    <t>The date/time at which the requested service should occur.</t>
+  </si>
+  <si>
+    <t>Request.occurrence[x]</t>
+  </si>
+  <si>
+    <t>TQ1/TQ2, OBR-7/OBR-8</t>
+  </si>
+  <si>
+    <t>.effectiveTime</t>
+  </si>
+  <si>
+    <t>FiveWs.planned</t>
+  </si>
+  <si>
+    <t>Procedure.procedureSchedule</t>
+  </si>
+  <si>
+    <t>ServiceRequest.asNeeded[x]</t>
+  </si>
+  <si>
+    <t>boolean
+CodeableConcept</t>
+  </si>
+  <si>
+    <t>Preconditions for service</t>
+  </si>
+  <si>
+    <t>If a CodeableConcept is present, it indicates the pre-condition for performing the service.  For example "pain", "on flare-up", etc.</t>
+  </si>
+  <si>
+    <t>A coded concept identifying the pre-condition that should hold prior to performing a procedure.  For example "pain", "on flare-up", etc.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/medication-as-needed-reason|4.0.1</t>
+  </si>
+  <si>
+    <t>boolean: precondition.negationInd (inversed - so negationInd = true means asNeeded=false CodeableConcept: precondition.observationEventCriterion[code="Assertion"].value</t>
+  </si>
+  <si>
+    <t>Proposal.prnReason.reason</t>
+  </si>
+  <si>
+    <t>ServiceRequest.authoredOn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">orderedOn
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dateTime
+</t>
+  </si>
+  <si>
+    <t>Date request signed</t>
+  </si>
+  <si>
+    <t>When the request transitioned to being actionable.</t>
+  </si>
+  <si>
+    <t>Request.authoredOn</t>
+  </si>
+  <si>
+    <t>ORC.9,  RF1-7 / RF1-9</t>
+  </si>
+  <si>
+    <t>.participation[typeCode=AUT].time</t>
+  </si>
+  <si>
+    <t>FiveWs.recorded</t>
+  </si>
+  <si>
+    <t>Proposal.proposedAtTime</t>
+  </si>
+  <si>
+    <t>ServiceRequest.requester</t>
+  </si>
+  <si>
+    <t>author
+orderer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(Practitioner|4.0.1|PractitionerRole|4.0.1|Organization|4.0.1|Patient|4.0.1|RelatedPerson|4.0.1|Device|4.0.1)
+</t>
+  </si>
+  <si>
+    <t>Who/what is requesting service</t>
+  </si>
+  <si>
+    <t>The individual who initiated the request and has responsibility for its activation.</t>
+  </si>
+  <si>
+    <t>This not the dispatcher, but rather who is the authorizer.  This element is not intended to handle delegation which would generally be managed through the Provenance resource.</t>
+  </si>
+  <si>
+    <t>Request.requester</t>
+  </si>
+  <si>
+    <t>ORC.12, PRT</t>
+  </si>
+  <si>
+    <t>.participation[typeCode=AUT].role</t>
+  </si>
+  <si>
+    <t>FiveWs.author</t>
+  </si>
+  <si>
+    <t>ClinicalStatement.statementAuthor</t>
+  </si>
+  <si>
+    <t>ServiceRequest.performerType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">specialty
+</t>
+  </si>
+  <si>
+    <t>Performer role</t>
+  </si>
+  <si>
+    <t>Desired type of performer for doing the requested service.</t>
+  </si>
+  <si>
+    <t>This is a  role, not  a participation type.  In other words, does not describe the task but describes the capacity.  For example, “compounding pharmacy”, “psychiatrist” or “internal referral”.</t>
+  </si>
+  <si>
+    <t>Indicates specific responsibility of an individual within the care team, such as "Primary physician", "Team coordinator", "Caregiver", etc.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/participant-role|4.0.1</t>
+  </si>
+  <si>
+    <t>Request.performerType</t>
+  </si>
+  <si>
+    <t>PRT, RF!-3</t>
+  </si>
+  <si>
+    <t>.participation[typeCode=PRF].role[scoper.determinerCode=KIND].code</t>
+  </si>
+  <si>
+    <t>FiveWs.actor</t>
+  </si>
+  <si>
+    <t>ServiceRequest.performer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">request recipient
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(Practitioner|4.0.1|PractitionerRole|4.0.1|Organization|4.0.1|CareTeam|4.0.1|HealthcareService|4.0.1|Patient|4.0.1|Device|4.0.1|RelatedPerson|4.0.1)
+</t>
+  </si>
+  <si>
+    <t>Requested performer</t>
+  </si>
+  <si>
+    <t>The desired performer for doing the requested service.  For example, the surgeon, dermatopathologist, endoscopist, etc.</t>
+  </si>
+  <si>
+    <t>If multiple performers are present, it is interpreted as a list of *alternative* performers without any preference regardless of order.  If order of preference is needed use the [request-performerOrder extension](http://hl7.org/fhir/R4/extension-request-performerorder.html).  Use CareTeam to represent a group of performers (for example, Practitioner A *and* Practitioner B).</t>
+  </si>
+  <si>
+    <t>Request.performer</t>
+  </si>
+  <si>
+    <t>PRT, Practitioner: PRD-2/PRD-7 where PRD-3 = RT; Organization: PRD-10 where PRD-3 = RT</t>
+  </si>
+  <si>
+    <t>.participation[typeCode=PRF].role[scoper.determinerCode=INSTANCE]</t>
+  </si>
+  <si>
+    <t>ServiceRequest.locationCode</t>
+  </si>
+  <si>
+    <t>Requested location</t>
+  </si>
+  <si>
+    <t>The preferred location(s) where the procedure should actually happen in coded or free text form. E.g. at home or nursing day care center.</t>
+  </si>
+  <si>
+    <t>A location type where services are delivered.</t>
+  </si>
+  <si>
+    <t>http://terminology.hl7.org/ValueSet/v3-ServiceDeliveryLocationRoleType|3.0.0</t>
+  </si>
+  <si>
+    <t>.participation[typeCode=LOC].role[scoper.determinerCode=KIND].code</t>
+  </si>
+  <si>
+    <t>ServiceRequest.locationReference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(Location|4.0.1)
+</t>
+  </si>
+  <si>
+    <t>A reference to the the preferred location(s) where the procedure should actually happen. E.g. at home or nursing day care center.</t>
+  </si>
+  <si>
+    <t>.participation[typeCode=LOC].role[scoper.determinerCode=INSTANCE]</t>
+  </si>
+  <si>
+    <t>ServiceRequest.reasonCode</t>
+  </si>
+  <si>
+    <t>Explanation/Justification for procedure or service</t>
+  </si>
+  <si>
+    <t>An explanation or justification for why this service is being requested in coded or textual form.   This is often for billing purposes.  May relate to the resources referred to in `supportingInfo`.</t>
+  </si>
+  <si>
+    <t>This element represents why the referral is being made and may be used to decide how the service will be performed, or even if it will be performed at all.   Use `CodeableConcept.text` element if the data is free (uncoded) text as shown in the [CT Scan example](http://hl7.org/fhir/R4/servicerequest-example-di.html).</t>
+  </si>
+  <si>
+    <t>Diagnosis or problem codes justifying the reason for requesting the service investigation.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/procedure-reason|4.0.1</t>
+  </si>
+  <si>
+    <t>Request.reasonCode</t>
+  </si>
+  <si>
+    <t>ORC.16, RF1-10</t>
+  </si>
+  <si>
+    <t>.reasonCode</t>
+  </si>
+  <si>
+    <t>FiveWs.why[x]</t>
+  </si>
+  <si>
+    <t>ServiceRequest.reasonReference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(Condition|4.0.1|Observation|4.0.1|DiagnosticReport|4.0.1|DocumentReference|4.0.1)
+</t>
+  </si>
+  <si>
+    <t>Explanation/Justification for service or service</t>
+  </si>
+  <si>
+    <t>Indicates another resource that provides a justification for why this service is being requested.   May relate to the resources referred to in `supportingInfo`.</t>
+  </si>
+  <si>
+    <t>This element represents why the referral is being made and may be used to decide how the service will be performed, or even if it will be performed at all.    To be as specific as possible,  a reference to  *Observation* or *Condition* should be used if available.  Otherwise when referencing  *DiagnosticReport*  it should contain a finding  in `DiagnosticReport.conclusion` and/or `DiagnosticReport.conclusionCode`.   When using a reference to *DocumentReference*, the target document should contain clear findings language providing the relevant reason for this service request.  Use  the CodeableConcept text element in `ServiceRequest.reasonCode` if the data is free (uncoded) text as shown in the [CT Scan example](http://hl7.org/fhir/R4/servicerequest-example-di.html).</t>
+  </si>
+  <si>
+    <t>Request.reasonReference</t>
+  </si>
+  <si>
+    <t>ORC.16</t>
+  </si>
+  <si>
+    <t>.outboundRelationship[typeCode=RSON].target</t>
+  </si>
+  <si>
+    <t>ServiceRequest.insurance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(Coverage|4.0.1|ClaimResponse|4.0.1)
+</t>
+  </si>
+  <si>
+    <t>Associated insurance coverage</t>
+  </si>
+  <si>
+    <t>Insurance plans, coverage extensions, pre-authorizations and/or pre-determinations that may be needed for delivering the requested service.</t>
+  </si>
+  <si>
+    <t>Request.insurance</t>
+  </si>
+  <si>
+    <t>IN1/IN2</t>
+  </si>
+  <si>
+    <t>.outboundRelationship[typeCode=COVBY].target</t>
+  </si>
+  <si>
+    <t>ServiceRequest.supportingInfo</t>
+  </si>
+  <si>
+    <t>Ask at order entry question
+AOE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(Resource|4.0.1)
+</t>
+  </si>
+  <si>
+    <t>Additional clinical information</t>
+  </si>
+  <si>
+    <t>Additional clinical information about the patient or specimen that may influence the services or their interpretations.     This information includes diagnosis, clinical findings and other observations.  In laboratory ordering these are typically referred to as "ask at order entry questions (AOEs)".  This includes observations explicitly requested by the producer (filler) to provide context or supporting information needed to complete the order. For example,  reporting the amount of inspired oxygen for blood gas measurements.</t>
+  </si>
+  <si>
+    <t>To represent information about how the services are to be delivered use the `instructions` element.</t>
+  </si>
+  <si>
+    <t>Request.supportingInfo</t>
+  </si>
+  <si>
+    <t>Accompanying segments</t>
+  </si>
+  <si>
+    <t>.outboundRelationship[typeCode=PERT].target</t>
+  </si>
+  <si>
+    <t>ServiceRequest.specimen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(Specimen|4.0.1)
+</t>
+  </si>
+  <si>
+    <t>Procedure Samples</t>
+  </si>
+  <si>
+    <t>One or more specimens that the laboratory procedure will use.</t>
+  </si>
+  <si>
+    <t>Many diagnostic procedures need a specimen, but the request itself is not actually about the specimen. This element is for when the diagnostic is requested on already existing specimens and the request points to the specimen it applies to.    Conversely, if the request is entered first with an unknown specimen, then the [Specimen](http://hl7.org/fhir/R4/specimen.html) resource points to the ServiceRequest.</t>
+  </si>
+  <si>
+    <t>SPM</t>
+  </si>
+  <si>
+    <t>.participation[typeCode=SPC].role</t>
+  </si>
+  <si>
+    <t>ServiceRequest.bodySite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location
+</t>
+  </si>
+  <si>
+    <t>Cible</t>
+  </si>
+  <si>
+    <t>Anatomic location where the procedure should be performed. This is the target site.</t>
+  </si>
+  <si>
+    <t>Only used if not implicit in the code found in ServiceRequest.code.  If the use case requires BodySite to be handled as a separate resource instead of an inline coded element (e.g. to identify and track separately)  then use the standard extension [procedure-targetBodyStructure](http://hl7.org/fhir/R4/extension-procedure-targetbodystructure.html).</t>
+  </si>
+  <si>
+    <t>Knowing where the procedure is performed is important for tracking if multiple sites are possible.</t>
+  </si>
+  <si>
+    <t>extensible</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/body-site|4.0.1</t>
+  </si>
+  <si>
+    <t>targetSiteCode</t>
+  </si>
+  <si>
+    <t>Procedure.targetBodySite</t>
+  </si>
+  <si>
+    <t>ServiceRequest.note</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annotation
+</t>
+  </si>
+  <si>
+    <t>Justification de la demande d'examen / Finalité de l'examen</t>
+  </si>
+  <si>
+    <t>Any other notes and comments made about the service request. For example, internal billing notes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value:text}
+</t>
+  </si>
+  <si>
+    <t>Request.note</t>
+  </si>
+  <si>
+    <t>.inboundRelationship(typeCode=SUBJ].source[classCode=ANNGEN, moodCode=EVN].value[xsi:type=ST]</t>
+  </si>
+  <si>
+    <t>ClinicalStatement.additionalText</t>
+  </si>
+  <si>
+    <t>ServiceRequest.note:finaliteExamen</t>
+  </si>
+  <si>
+    <t>finaliteExamen</t>
+  </si>
+  <si>
+    <t>Finalité de l'examen demandé</t>
+  </si>
+  <si>
+    <t>ServiceRequest.note:justificationDemande</t>
+  </si>
+  <si>
+    <t>justificationDemande</t>
+  </si>
+  <si>
+    <t>Justification de la demande d'examen</t>
+  </si>
+  <si>
+    <t>ServiceRequest.patientInstruction</t>
   </si>
   <si>
     <t xml:space="preserve">string
 </t>
-  </si>
-  <si>
-    <t>Unique id for inter-element referencing</t>
-  </si>
-  <si>
-    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
-  </si>
-  <si>
-    <t>Element.id</t>
-  </si>
-  <si>
-    <t>n/a</t>
-  </si>
-  <si>
-    <t>ServiceRequest.orderDetail.extension</t>
-  </si>
-  <si>
-    <t>Additional content defined by implementations</t>
-  </si>
-  <si>
-    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
-  </si>
-  <si>
-    <t>Extensions are always sliced by (at least) url</t>
-  </si>
-  <si>
-    <t>Element.extension</t>
-  </si>
-  <si>
-    <t>ServiceRequest.orderDetail.coding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coding
-</t>
-  </si>
-  <si>
-    <t>Résultat de la demande</t>
-  </si>
-  <si>
-    <t>A reference to a code defined by a terminology system.</t>
-  </si>
-  <si>
-    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
-  </si>
-  <si>
-    <t>Allows for alternative encodings within a code system, and translations to other code systems.</t>
-  </si>
-  <si>
-    <t>CodeableConcept.coding</t>
-  </si>
-  <si>
-    <t>C*E.1-8, C*E.10-22</t>
-  </si>
-  <si>
-    <t>union(., ./translation)</t>
-  </si>
-  <si>
-    <t>ServiceRequest.orderDetail.text</t>
-  </si>
-  <si>
-    <t>Plain text representation of the concept</t>
-  </si>
-  <si>
-    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
-  </si>
-  <si>
-    <t>Very often the text is the same as a displayName of one of the codings.</t>
-  </si>
-  <si>
-    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
-  </si>
-  <si>
-    <t>CodeableConcept.text</t>
-  </si>
-  <si>
-    <t>C*E.9. But note many systems use C*E.2 for this</t>
-  </si>
-  <si>
-    <t>./originalText[mediaType/code="text/plain"]/data</t>
-  </si>
-  <si>
-    <t>ServiceRequest.quantity[x]</t>
-  </si>
-  <si>
-    <t>Quantity
-RatioRange</t>
-  </si>
-  <si>
-    <t>Service amount</t>
-  </si>
-  <si>
-    <t>An amount of service being requested which can be a quantity ( for example $1,500 home modification), a ratio ( for example, 20 half day visits per month), or a range (2.0 to 1.8 Gy per fraction).</t>
-  </si>
-  <si>
-    <t>When ordering a service the number of service items may need to be specified separately from the the service item.</t>
-  </si>
-  <si>
-    <t>.quantity</t>
-  </si>
-  <si>
-    <t>ServiceRequest.subject</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(Patient|4.0.1|Group|4.0.1|Location|4.0.1|Device|4.0.1)
-</t>
-  </si>
-  <si>
-    <t>Individual or Entity the service is ordered for</t>
-  </si>
-  <si>
-    <t>On whom or what the service is to be performed. This is usually a human patient, but can also be requested on animals, groups of humans or animals, devices such as dialysis machines, or even locations (typically for environmental scans).</t>
-  </si>
-  <si>
-    <t>Request.subject</t>
-  </si>
-  <si>
-    <t>PID</t>
-  </si>
-  <si>
-    <t>.participation[typeCode=SBJ].role</t>
-  </si>
-  <si>
-    <t>FiveWs.subject</t>
-  </si>
-  <si>
-    <t>ClinicalStatement.subject</t>
-  </si>
-  <si>
-    <t>ServiceRequest.encounter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">context
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(Encounter|4.0.1)
-</t>
-  </si>
-  <si>
-    <t>Encounter in which the request was created</t>
-  </si>
-  <si>
-    <t>An encounter that provides additional information about the healthcare context in which this request is made.</t>
-  </si>
-  <si>
-    <t>Request.encounter</t>
-  </si>
-  <si>
-    <t>PV1</t>
-  </si>
-  <si>
-    <t>.inboundRelationship(typeCode=COMP].source[classCode&lt;=PCPR, moodCode=EVN]</t>
-  </si>
-  <si>
-    <t>FiveWs.context</t>
-  </si>
-  <si>
-    <t>ClinicalStatement.encounter</t>
-  </si>
-  <si>
-    <t>ServiceRequest.occurrence[x]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">schedule
-</t>
-  </si>
-  <si>
-    <t>dateTime
-PeriodTiming</t>
-  </si>
-  <si>
-    <t>Date prévisionnelle de l'examen, du suivi, de l'objectif</t>
-  </si>
-  <si>
-    <t>The date/time at which the requested service should occur.</t>
-  </si>
-  <si>
-    <t>Request.occurrence[x]</t>
-  </si>
-  <si>
-    <t>TQ1/TQ2, OBR-7/OBR-8</t>
-  </si>
-  <si>
-    <t>.effectiveTime</t>
-  </si>
-  <si>
-    <t>FiveWs.planned</t>
-  </si>
-  <si>
-    <t>Procedure.procedureSchedule</t>
-  </si>
-  <si>
-    <t>ServiceRequest.asNeeded[x]</t>
-  </si>
-  <si>
-    <t>boolean
-CodeableConcept</t>
-  </si>
-  <si>
-    <t>Preconditions for service</t>
-  </si>
-  <si>
-    <t>If a CodeableConcept is present, it indicates the pre-condition for performing the service.  For example "pain", "on flare-up", etc.</t>
-  </si>
-  <si>
-    <t>A coded concept identifying the pre-condition that should hold prior to performing a procedure.  For example "pain", "on flare-up", etc.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/medication-as-needed-reason|4.0.1</t>
-  </si>
-  <si>
-    <t>boolean: precondition.negationInd (inversed - so negationInd = true means asNeeded=false CodeableConcept: precondition.observationEventCriterion[code="Assertion"].value</t>
-  </si>
-  <si>
-    <t>Proposal.prnReason.reason</t>
-  </si>
-  <si>
-    <t>ServiceRequest.authoredOn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">orderedOn
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dateTime
-</t>
-  </si>
-  <si>
-    <t>Date request signed</t>
-  </si>
-  <si>
-    <t>When the request transitioned to being actionable.</t>
-  </si>
-  <si>
-    <t>Request.authoredOn</t>
-  </si>
-  <si>
-    <t>ORC.9,  RF1-7 / RF1-9</t>
-  </si>
-  <si>
-    <t>.participation[typeCode=AUT].time</t>
-  </si>
-  <si>
-    <t>FiveWs.recorded</t>
-  </si>
-  <si>
-    <t>Proposal.proposedAtTime</t>
-  </si>
-  <si>
-    <t>ServiceRequest.requester</t>
-  </si>
-  <si>
-    <t>author
-orderer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(Practitioner|4.0.1|PractitionerRole|4.0.1|Organization|4.0.1|Patient|4.0.1|RelatedPerson|4.0.1|Device|4.0.1)
-</t>
-  </si>
-  <si>
-    <t>Who/what is requesting service</t>
-  </si>
-  <si>
-    <t>The individual who initiated the request and has responsibility for its activation.</t>
-  </si>
-  <si>
-    <t>This not the dispatcher, but rather who is the authorizer.  This element is not intended to handle delegation which would generally be managed through the Provenance resource.</t>
-  </si>
-  <si>
-    <t>Request.requester</t>
-  </si>
-  <si>
-    <t>ORC.12, PRT</t>
-  </si>
-  <si>
-    <t>.participation[typeCode=AUT].role</t>
-  </si>
-  <si>
-    <t>FiveWs.author</t>
-  </si>
-  <si>
-    <t>ClinicalStatement.statementAuthor</t>
-  </si>
-  <si>
-    <t>ServiceRequest.performerType</t>
-  </si>
-  <si>
-    <t xml:space="preserve">specialty
-</t>
-  </si>
-  <si>
-    <t>Performer role</t>
-  </si>
-  <si>
-    <t>Desired type of performer for doing the requested service.</t>
-  </si>
-  <si>
-    <t>This is a  role, not  a participation type.  In other words, does not describe the task but describes the capacity.  For example, “compounding pharmacy”, “psychiatrist” or “internal referral”.</t>
-  </si>
-  <si>
-    <t>Indicates specific responsibility of an individual within the care team, such as "Primary physician", "Team coordinator", "Caregiver", etc.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/participant-role|4.0.1</t>
-  </si>
-  <si>
-    <t>Request.performerType</t>
-  </si>
-  <si>
-    <t>PRT, RF!-3</t>
-  </si>
-  <si>
-    <t>.participation[typeCode=PRF].role[scoper.determinerCode=KIND].code</t>
-  </si>
-  <si>
-    <t>FiveWs.actor</t>
-  </si>
-  <si>
-    <t>ServiceRequest.performer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">request recipient
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(Practitioner|4.0.1|PractitionerRole|4.0.1|Organization|4.0.1|CareTeam|4.0.1|HealthcareService|4.0.1|Patient|4.0.1|Device|4.0.1|RelatedPerson|4.0.1)
-</t>
-  </si>
-  <si>
-    <t>Requested performer</t>
-  </si>
-  <si>
-    <t>The desired performer for doing the requested service.  For example, the surgeon, dermatopathologist, endoscopist, etc.</t>
-  </si>
-  <si>
-    <t>If multiple performers are present, it is interpreted as a list of *alternative* performers without any preference regardless of order.  If order of preference is needed use the [request-performerOrder extension](http://hl7.org/fhir/R4/extension-request-performerorder.html).  Use CareTeam to represent a group of performers (for example, Practitioner A *and* Practitioner B).</t>
-  </si>
-  <si>
-    <t>Request.performer</t>
-  </si>
-  <si>
-    <t>PRT, Practitioner: PRD-2/PRD-7 where PRD-3 = RT; Organization: PRD-10 where PRD-3 = RT</t>
-  </si>
-  <si>
-    <t>.participation[typeCode=PRF].role[scoper.determinerCode=INSTANCE]</t>
-  </si>
-  <si>
-    <t>ServiceRequest.locationCode</t>
-  </si>
-  <si>
-    <t>Requested location</t>
-  </si>
-  <si>
-    <t>The preferred location(s) where the procedure should actually happen in coded or free text form. E.g. at home or nursing day care center.</t>
-  </si>
-  <si>
-    <t>A location type where services are delivered.</t>
-  </si>
-  <si>
-    <t>http://terminology.hl7.org/ValueSet/v3-ServiceDeliveryLocationRoleType|3.0.0</t>
-  </si>
-  <si>
-    <t>.participation[typeCode=LOC].role[scoper.determinerCode=KIND].code</t>
-  </si>
-  <si>
-    <t>ServiceRequest.locationReference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(Location|4.0.1)
-</t>
-  </si>
-  <si>
-    <t>A reference to the the preferred location(s) where the procedure should actually happen. E.g. at home or nursing day care center.</t>
-  </si>
-  <si>
-    <t>.participation[typeCode=LOC].role[scoper.determinerCode=INSTANCE]</t>
-  </si>
-  <si>
-    <t>ServiceRequest.reasonCode</t>
-  </si>
-  <si>
-    <t>Explanation/Justification for procedure or service</t>
-  </si>
-  <si>
-    <t>An explanation or justification for why this service is being requested in coded or textual form.   This is often for billing purposes.  May relate to the resources referred to in `supportingInfo`.</t>
-  </si>
-  <si>
-    <t>This element represents why the referral is being made and may be used to decide how the service will be performed, or even if it will be performed at all.   Use `CodeableConcept.text` element if the data is free (uncoded) text as shown in the [CT Scan example](http://hl7.org/fhir/R4/servicerequest-example-di.html).</t>
-  </si>
-  <si>
-    <t>Diagnosis or problem codes justifying the reason for requesting the service investigation.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/procedure-reason|4.0.1</t>
-  </si>
-  <si>
-    <t>Request.reasonCode</t>
-  </si>
-  <si>
-    <t>ORC.16, RF1-10</t>
-  </si>
-  <si>
-    <t>.reasonCode</t>
-  </si>
-  <si>
-    <t>FiveWs.why[x]</t>
-  </si>
-  <si>
-    <t>ServiceRequest.reasonReference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(Condition|4.0.1|Observation|4.0.1|DiagnosticReport|4.0.1|DocumentReference|4.0.1)
-</t>
-  </si>
-  <si>
-    <t>Explanation/Justification for service or service</t>
-  </si>
-  <si>
-    <t>Indicates another resource that provides a justification for why this service is being requested.   May relate to the resources referred to in `supportingInfo`.</t>
-  </si>
-  <si>
-    <t>This element represents why the referral is being made and may be used to decide how the service will be performed, or even if it will be performed at all.    To be as specific as possible,  a reference to  *Observation* or *Condition* should be used if available.  Otherwise when referencing  *DiagnosticReport*  it should contain a finding  in `DiagnosticReport.conclusion` and/or `DiagnosticReport.conclusionCode`.   When using a reference to *DocumentReference*, the target document should contain clear findings language providing the relevant reason for this service request.  Use  the CodeableConcept text element in `ServiceRequest.reasonCode` if the data is free (uncoded) text as shown in the [CT Scan example](http://hl7.org/fhir/R4/servicerequest-example-di.html).</t>
-  </si>
-  <si>
-    <t>Request.reasonReference</t>
-  </si>
-  <si>
-    <t>ORC.16</t>
-  </si>
-  <si>
-    <t>.outboundRelationship[typeCode=RSON].target</t>
-  </si>
-  <si>
-    <t>ServiceRequest.insurance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(Coverage|4.0.1|ClaimResponse|4.0.1)
-</t>
-  </si>
-  <si>
-    <t>Associated insurance coverage</t>
-  </si>
-  <si>
-    <t>Insurance plans, coverage extensions, pre-authorizations and/or pre-determinations that may be needed for delivering the requested service.</t>
-  </si>
-  <si>
-    <t>Request.insurance</t>
-  </si>
-  <si>
-    <t>IN1/IN2</t>
-  </si>
-  <si>
-    <t>.outboundRelationship[typeCode=COVBY].target</t>
-  </si>
-  <si>
-    <t>ServiceRequest.supportingInfo</t>
-  </si>
-  <si>
-    <t>Ask at order entry question
-AOE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(Resource|4.0.1)
-</t>
-  </si>
-  <si>
-    <t>Additional clinical information</t>
-  </si>
-  <si>
-    <t>Additional clinical information about the patient or specimen that may influence the services or their interpretations.     This information includes diagnosis, clinical findings and other observations.  In laboratory ordering these are typically referred to as "ask at order entry questions (AOEs)".  This includes observations explicitly requested by the producer (filler) to provide context or supporting information needed to complete the order. For example,  reporting the amount of inspired oxygen for blood gas measurements.</t>
-  </si>
-  <si>
-    <t>To represent information about how the services are to be delivered use the `instructions` element.</t>
-  </si>
-  <si>
-    <t>Request.supportingInfo</t>
-  </si>
-  <si>
-    <t>Accompanying segments</t>
-  </si>
-  <si>
-    <t>.outboundRelationship[typeCode=PERT].target</t>
-  </si>
-  <si>
-    <t>ServiceRequest.specimen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(Specimen|4.0.1)
-</t>
-  </si>
-  <si>
-    <t>Procedure Samples</t>
-  </si>
-  <si>
-    <t>One or more specimens that the laboratory procedure will use.</t>
-  </si>
-  <si>
-    <t>Many diagnostic procedures need a specimen, but the request itself is not actually about the specimen. This element is for when the diagnostic is requested on already existing specimens and the request points to the specimen it applies to.    Conversely, if the request is entered first with an unknown specimen, then the [Specimen](http://hl7.org/fhir/R4/specimen.html) resource points to the ServiceRequest.</t>
-  </si>
-  <si>
-    <t>SPM</t>
-  </si>
-  <si>
-    <t>.participation[typeCode=SPC].role</t>
-  </si>
-  <si>
-    <t>ServiceRequest.bodySite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">location
-</t>
-  </si>
-  <si>
-    <t>Cible</t>
-  </si>
-  <si>
-    <t>Anatomic location where the procedure should be performed. This is the target site.</t>
-  </si>
-  <si>
-    <t>Only used if not implicit in the code found in ServiceRequest.code.  If the use case requires BodySite to be handled as a separate resource instead of an inline coded element (e.g. to identify and track separately)  then use the standard extension [procedure-targetBodyStructure](http://hl7.org/fhir/R4/extension-procedure-targetbodystructure.html).</t>
-  </si>
-  <si>
-    <t>Knowing where the procedure is performed is important for tracking if multiple sites are possible.</t>
-  </si>
-  <si>
-    <t>extensible</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/body-site|4.0.1</t>
-  </si>
-  <si>
-    <t>targetSiteCode</t>
-  </si>
-  <si>
-    <t>Procedure.targetBodySite</t>
-  </si>
-  <si>
-    <t>ServiceRequest.note</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annotation
-</t>
-  </si>
-  <si>
-    <t>Justification de la demande d'examen / Finalité de l'examen</t>
-  </si>
-  <si>
-    <t>Any other notes and comments made about the service request. For example, internal billing notes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value:text}
-</t>
-  </si>
-  <si>
-    <t>Request.note</t>
-  </si>
-  <si>
-    <t>.inboundRelationship(typeCode=SUBJ].source[classCode=ANNGEN, moodCode=EVN].value[xsi:type=ST]</t>
-  </si>
-  <si>
-    <t>ClinicalStatement.additionalText</t>
-  </si>
-  <si>
-    <t>ServiceRequest.note:finaliteExamen</t>
-  </si>
-  <si>
-    <t>finaliteExamen</t>
-  </si>
-  <si>
-    <t>Finalité de l'examen demandé</t>
-  </si>
-  <si>
-    <t>ServiceRequest.note:justificationDemande</t>
-  </si>
-  <si>
-    <t>justificationDemande</t>
-  </si>
-  <si>
-    <t>Justification de la demande d'examen</t>
-  </si>
-  <si>
-    <t>ServiceRequest.patientInstruction</t>
   </si>
   <si>
     <t>Patient or consumer-oriented instructions</t>
@@ -1823,11 +1741,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AO51"/>
+  <dimension ref="A1:AO47"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="35.24609375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="30.69921875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="30.62109375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="17.66015625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="37.7265625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -1854,7 +1772,7 @@
     <col min="26" max="26" width="62.65234375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="32" max="32" width="30.62109375" customWidth="true" bestFit="true" hidden="true"/>
@@ -4698,7 +4616,7 @@
         <v>80</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>82</v>
@@ -4824,7 +4742,7 @@
         <v>82</v>
       </c>
       <c r="J26" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="K26" t="s" s="2">
         <v>282</v>
@@ -4836,7 +4754,9 @@
         <v>284</v>
       </c>
       <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
+      <c r="O26" t="s" s="2">
+        <v>285</v>
+      </c>
       <c r="P26" t="s" s="2">
         <v>82</v>
       </c>
@@ -4884,7 +4804,7 @@
         <v>82</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>80</v>
@@ -4896,13 +4816,13 @@
         <v>82</v>
       </c>
       <c r="AJ26" t="s" s="2">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="AK26" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>82</v>
+        <v>280</v>
       </c>
       <c r="AM26" t="s" s="2">
         <v>286</v>
@@ -4923,14 +4843,14 @@
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>150</v>
+        <v>82</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H27" t="s" s="2">
         <v>82</v>
@@ -4939,20 +4859,18 @@
         <v>82</v>
       </c>
       <c r="J27" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>136</v>
+        <v>288</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>289</v>
-      </c>
-      <c r="N27" t="s" s="2">
-        <v>153</v>
-      </c>
+        <v>290</v>
+      </c>
+      <c r="N27" s="2"/>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
         <v>82</v>
@@ -4989,65 +4907,65 @@
         <v>82</v>
       </c>
       <c r="AB27" t="s" s="2">
-        <v>139</v>
+        <v>82</v>
       </c>
       <c r="AC27" t="s" s="2">
-        <v>290</v>
+        <v>82</v>
       </c>
       <c r="AD27" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE27" t="s" s="2">
-        <v>140</v>
+        <v>82</v>
       </c>
       <c r="AF27" t="s" s="2">
+        <v>287</v>
+      </c>
+      <c r="AG27" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AH27" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ27" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AK27" t="s" s="2">
         <v>291</v>
       </c>
-      <c r="AG27" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH27" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI27" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ27" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="AK27" t="s" s="2">
-        <v>82</v>
-      </c>
       <c r="AL27" t="s" s="2">
-        <v>82</v>
+        <v>292</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="AN27" t="s" s="2">
-        <v>82</v>
+        <v>294</v>
       </c>
       <c r="AO27" t="s" s="2">
-        <v>82</v>
+        <v>295</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
-        <v>82</v>
+        <v>297</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>82</v>
@@ -5059,20 +4977,16 @@
         <v>92</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>295</v>
-      </c>
-      <c r="N28" t="s" s="2">
-        <v>296</v>
-      </c>
-      <c r="O28" t="s" s="2">
-        <v>297</v>
-      </c>
+        <v>300</v>
+      </c>
+      <c r="N28" s="2"/>
+      <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>82</v>
       </c>
@@ -5120,13 +5034,13 @@
         <v>82</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>82</v>
@@ -5135,35 +5049,35 @@
         <v>103</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>82</v>
+        <v>301</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>82</v>
+        <v>304</v>
       </c>
       <c r="AO28" t="s" s="2">
-        <v>82</v>
+        <v>305</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
-        <v>82</v>
+        <v>307</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="G29" t="s" s="2">
         <v>91</v>
@@ -5178,20 +5092,16 @@
         <v>92</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>282</v>
+        <v>308</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>303</v>
-      </c>
-      <c r="N29" t="s" s="2">
-        <v>304</v>
-      </c>
-      <c r="O29" t="s" s="2">
-        <v>305</v>
-      </c>
+        <v>310</v>
+      </c>
+      <c r="N29" s="2"/>
+      <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
         <v>82</v>
       </c>
@@ -5254,27 +5164,27 @@
         <v>103</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>82</v>
+        <v>311</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>82</v>
+        <v>314</v>
       </c>
       <c r="AO29" t="s" s="2">
-        <v>82</v>
+        <v>315</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5297,18 +5207,16 @@
         <v>92</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="N30" s="2"/>
-      <c r="O30" t="s" s="2">
-        <v>313</v>
-      </c>
+      <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>82</v>
       </c>
@@ -5332,13 +5240,13 @@
         <v>82</v>
       </c>
       <c r="X30" t="s" s="2">
-        <v>82</v>
+        <v>236</v>
       </c>
       <c r="Y30" t="s" s="2">
-        <v>82</v>
+        <v>320</v>
       </c>
       <c r="Z30" t="s" s="2">
-        <v>82</v>
+        <v>321</v>
       </c>
       <c r="AA30" t="s" s="2">
         <v>82</v>
@@ -5356,7 +5264,7 @@
         <v>82</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>80</v>
@@ -5374,32 +5282,32 @@
         <v>82</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>280</v>
+        <v>82</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="AN30" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO30" t="s" s="2">
-        <v>82</v>
+        <v>323</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>82</v>
+        <v>325</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G31" t="s" s="2">
         <v>91</v>
@@ -5414,13 +5322,13 @@
         <v>92</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>316</v>
+        <v>326</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>317</v>
+        <v>327</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>318</v>
+        <v>328</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -5471,10 +5379,10 @@
         <v>82</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="AG31" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="AH31" t="s" s="2">
         <v>91</v>
@@ -5486,31 +5394,31 @@
         <v>103</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>319</v>
+        <v>329</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>320</v>
+        <v>330</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>321</v>
+        <v>331</v>
       </c>
       <c r="AN31" t="s" s="2">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="AO31" t="s" s="2">
-        <v>323</v>
+        <v>333</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>324</v>
+        <v>334</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>324</v>
+        <v>334</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>325</v>
+        <v>335</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
@@ -5529,15 +5437,17 @@
         <v>92</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>328</v>
-      </c>
-      <c r="N32" s="2"/>
+        <v>338</v>
+      </c>
+      <c r="N32" t="s" s="2">
+        <v>339</v>
+      </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
         <v>82</v>
@@ -5586,7 +5496,7 @@
         <v>82</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>324</v>
+        <v>334</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>80</v>
@@ -5601,35 +5511,35 @@
         <v>103</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>329</v>
+        <v>340</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>330</v>
+        <v>341</v>
       </c>
       <c r="AM32" t="s" s="2">
-        <v>331</v>
+        <v>342</v>
       </c>
       <c r="AN32" t="s" s="2">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="AO32" t="s" s="2">
-        <v>333</v>
+        <v>344</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>334</v>
+        <v>345</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>334</v>
+        <v>345</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>335</v>
+        <v>346</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G33" t="s" s="2">
         <v>91</v>
@@ -5644,15 +5554,17 @@
         <v>92</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>336</v>
+        <v>231</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>337</v>
+        <v>347</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>338</v>
-      </c>
-      <c r="N33" s="2"/>
+        <v>348</v>
+      </c>
+      <c r="N33" t="s" s="2">
+        <v>349</v>
+      </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
         <v>82</v>
@@ -5677,13 +5589,13 @@
         <v>82</v>
       </c>
       <c r="X33" t="s" s="2">
-        <v>82</v>
+        <v>236</v>
       </c>
       <c r="Y33" t="s" s="2">
-        <v>82</v>
+        <v>350</v>
       </c>
       <c r="Z33" t="s" s="2">
-        <v>82</v>
+        <v>351</v>
       </c>
       <c r="AA33" t="s" s="2">
         <v>82</v>
@@ -5701,7 +5613,7 @@
         <v>82</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>334</v>
+        <v>345</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>80</v>
@@ -5716,38 +5628,38 @@
         <v>103</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>339</v>
+        <v>352</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>340</v>
+        <v>353</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>341</v>
+        <v>354</v>
       </c>
       <c r="AN33" t="s" s="2">
-        <v>342</v>
+        <v>355</v>
       </c>
       <c r="AO33" t="s" s="2">
-        <v>343</v>
+        <v>82</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>82</v>
+        <v>357</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>82</v>
@@ -5759,15 +5671,17 @@
         <v>92</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>345</v>
+        <v>358</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>346</v>
+        <v>359</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>347</v>
-      </c>
-      <c r="N34" s="2"/>
+        <v>360</v>
+      </c>
+      <c r="N34" t="s" s="2">
+        <v>361</v>
+      </c>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>82</v>
@@ -5792,13 +5706,13 @@
         <v>82</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>236</v>
+        <v>82</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>348</v>
+        <v>82</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>349</v>
+        <v>82</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>82</v>
@@ -5816,13 +5730,13 @@
         <v>82</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH34" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI34" t="s" s="2">
         <v>82</v>
@@ -5831,38 +5745,38 @@
         <v>103</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>82</v>
+        <v>362</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>82</v>
+        <v>363</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>350</v>
+        <v>364</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>82</v>
+        <v>355</v>
       </c>
       <c r="AO34" t="s" s="2">
-        <v>351</v>
+        <v>82</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>352</v>
+        <v>365</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>352</v>
+        <v>365</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
-        <v>353</v>
+        <v>82</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>82</v>
@@ -5874,13 +5788,13 @@
         <v>92</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>354</v>
+        <v>231</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>355</v>
+        <v>366</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>356</v>
+        <v>367</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -5907,13 +5821,13 @@
         <v>82</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>82</v>
+        <v>236</v>
       </c>
       <c r="Y35" t="s" s="2">
-        <v>82</v>
+        <v>368</v>
       </c>
       <c r="Z35" t="s" s="2">
-        <v>82</v>
+        <v>369</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>82</v>
@@ -5931,13 +5845,13 @@
         <v>82</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>352</v>
+        <v>365</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI35" t="s" s="2">
         <v>82</v>
@@ -5946,38 +5860,38 @@
         <v>103</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>357</v>
+        <v>82</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>358</v>
+        <v>82</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>359</v>
+        <v>370</v>
       </c>
       <c r="AN35" t="s" s="2">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="AO35" t="s" s="2">
-        <v>361</v>
+        <v>82</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>362</v>
+        <v>371</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>362</v>
+        <v>371</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
-        <v>363</v>
+        <v>82</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H36" t="s" s="2">
         <v>82</v>
@@ -5989,17 +5903,15 @@
         <v>92</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>366</v>
-      </c>
-      <c r="N36" t="s" s="2">
-        <v>367</v>
-      </c>
+        <v>373</v>
+      </c>
+      <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>82</v>
@@ -6048,13 +5960,13 @@
         <v>82</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>362</v>
+        <v>371</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>82</v>
@@ -6063,38 +5975,38 @@
         <v>103</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>368</v>
+        <v>82</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>369</v>
+        <v>82</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>371</v>
+        <v>355</v>
       </c>
       <c r="AO36" t="s" s="2">
-        <v>372</v>
+        <v>82</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>374</v>
+        <v>82</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>82</v>
@@ -6109,13 +6021,13 @@
         <v>231</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -6144,10 +6056,10 @@
         <v>236</v>
       </c>
       <c r="Y37" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="Z37" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="AA37" t="s" s="2">
         <v>82</v>
@@ -6165,13 +6077,13 @@
         <v>82</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>82</v>
@@ -6180,16 +6092,16 @@
         <v>103</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AO37" t="s" s="2">
         <v>82</v>
@@ -6197,14 +6109,14 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>385</v>
+        <v>82</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
@@ -6282,7 +6194,7 @@
         <v>82</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>80</v>
@@ -6306,7 +6218,7 @@
         <v>392</v>
       </c>
       <c r="AN38" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AO38" t="s" s="2">
         <v>82</v>
@@ -6337,16 +6249,16 @@
         <v>82</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>231</v>
+        <v>394</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -6373,13 +6285,13 @@
         <v>82</v>
       </c>
       <c r="X39" t="s" s="2">
-        <v>236</v>
+        <v>82</v>
       </c>
       <c r="Y39" t="s" s="2">
-        <v>396</v>
+        <v>82</v>
       </c>
       <c r="Z39" t="s" s="2">
-        <v>397</v>
+        <v>82</v>
       </c>
       <c r="AA39" t="s" s="2">
         <v>82</v>
@@ -6412,16 +6324,16 @@
         <v>103</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>82</v>
+        <v>397</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>82</v>
+        <v>398</v>
       </c>
       <c r="AM39" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="AN39" t="s" s="2">
-        <v>383</v>
+        <v>82</v>
       </c>
       <c r="AO39" t="s" s="2">
         <v>82</v>
@@ -6429,14 +6341,14 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
-        <v>82</v>
+        <v>401</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
@@ -6452,18 +6364,20 @@
         <v>82</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>394</v>
+        <v>403</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>401</v>
-      </c>
-      <c r="N40" s="2"/>
+        <v>404</v>
+      </c>
+      <c r="N40" t="s" s="2">
+        <v>405</v>
+      </c>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>82</v>
@@ -6512,7 +6426,7 @@
         <v>82</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>80</v>
@@ -6527,16 +6441,16 @@
         <v>103</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>82</v>
+        <v>406</v>
       </c>
       <c r="AL40" t="s" s="2">
-        <v>82</v>
+        <v>407</v>
       </c>
       <c r="AM40" t="s" s="2">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>383</v>
+        <v>82</v>
       </c>
       <c r="AO40" t="s" s="2">
         <v>82</v>
@@ -6544,10 +6458,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6570,16 +6484,16 @@
         <v>92</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>231</v>
+        <v>410</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="N41" t="s" s="2">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
@@ -6605,13 +6519,13 @@
         <v>82</v>
       </c>
       <c r="X41" t="s" s="2">
-        <v>236</v>
+        <v>82</v>
       </c>
       <c r="Y41" t="s" s="2">
-        <v>407</v>
+        <v>82</v>
       </c>
       <c r="Z41" t="s" s="2">
-        <v>408</v>
+        <v>82</v>
       </c>
       <c r="AA41" t="s" s="2">
         <v>82</v>
@@ -6629,7 +6543,7 @@
         <v>82</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>80</v>
@@ -6644,16 +6558,16 @@
         <v>103</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>409</v>
+        <v>82</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="AN41" t="s" s="2">
-        <v>412</v>
+        <v>82</v>
       </c>
       <c r="AO41" t="s" s="2">
         <v>82</v>
@@ -6661,14 +6575,14 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>82</v>
+        <v>417</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
@@ -6687,18 +6601,20 @@
         <v>92</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>414</v>
+        <v>231</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="N42" t="s" s="2">
-        <v>417</v>
-      </c>
-      <c r="O42" s="2"/>
+        <v>420</v>
+      </c>
+      <c r="O42" t="s" s="2">
+        <v>421</v>
+      </c>
       <c r="P42" t="s" s="2">
         <v>82</v>
       </c>
@@ -6722,13 +6638,11 @@
         <v>82</v>
       </c>
       <c r="X42" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y42" t="s" s="2">
-        <v>82</v>
-      </c>
+        <v>422</v>
+      </c>
+      <c r="Y42" s="2"/>
       <c r="Z42" t="s" s="2">
-        <v>82</v>
+        <v>423</v>
       </c>
       <c r="AA42" t="s" s="2">
         <v>82</v>
@@ -6746,7 +6660,7 @@
         <v>82</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>80</v>
@@ -6761,27 +6675,27 @@
         <v>103</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>418</v>
+        <v>82</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>412</v>
+        <v>82</v>
       </c>
       <c r="AO42" t="s" s="2">
-        <v>82</v>
+        <v>425</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6789,7 +6703,7 @@
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
-        <v>80</v>
+        <v>427</v>
       </c>
       <c r="G43" t="s" s="2">
         <v>81</v>
@@ -6804,13 +6718,13 @@
         <v>82</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>422</v>
+        <v>428</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>423</v>
+        <v>429</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -6849,19 +6763,17 @@
         <v>82</v>
       </c>
       <c r="AB43" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC43" t="s" s="2">
-        <v>82</v>
-      </c>
+        <v>431</v>
+      </c>
+      <c r="AC43" s="2"/>
       <c r="AD43" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE43" t="s" s="2">
-        <v>82</v>
+        <v>140</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>80</v>
@@ -6876,38 +6788,40 @@
         <v>103</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>426</v>
+        <v>280</v>
       </c>
       <c r="AM43" t="s" s="2">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="AN43" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO43" t="s" s="2">
-        <v>82</v>
+        <v>434</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>428</v>
-      </c>
-      <c r="C44" s="2"/>
+        <v>426</v>
+      </c>
+      <c r="C44" t="s" s="2">
+        <v>436</v>
+      </c>
       <c r="D44" t="s" s="2">
-        <v>429</v>
+        <v>82</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>82</v>
@@ -6919,17 +6833,15 @@
         <v>82</v>
       </c>
       <c r="K44" t="s" s="2">
+        <v>428</v>
+      </c>
+      <c r="L44" t="s" s="2">
+        <v>437</v>
+      </c>
+      <c r="M44" t="s" s="2">
         <v>430</v>
       </c>
-      <c r="L44" t="s" s="2">
-        <v>431</v>
-      </c>
-      <c r="M44" t="s" s="2">
-        <v>432</v>
-      </c>
-      <c r="N44" t="s" s="2">
-        <v>433</v>
-      </c>
+      <c r="N44" s="2"/>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
         <v>82</v>
@@ -6978,7 +6890,7 @@
         <v>82</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>80</v>
@@ -6993,38 +6905,40 @@
         <v>103</v>
       </c>
       <c r="AK44" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="AL44" t="s" s="2">
+        <v>280</v>
+      </c>
+      <c r="AM44" t="s" s="2">
+        <v>433</v>
+      </c>
+      <c r="AN44" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO44" t="s" s="2">
         <v>434</v>
-      </c>
-      <c r="AL44" t="s" s="2">
-        <v>435</v>
-      </c>
-      <c r="AM44" t="s" s="2">
-        <v>436</v>
-      </c>
-      <c r="AN44" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO44" t="s" s="2">
-        <v>82</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>437</v>
-      </c>
-      <c r="C45" s="2"/>
+        <v>426</v>
+      </c>
+      <c r="C45" t="s" s="2">
+        <v>439</v>
+      </c>
       <c r="D45" t="s" s="2">
         <v>82</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H45" t="s" s="2">
         <v>82</v>
@@ -7033,20 +6947,18 @@
         <v>82</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>438</v>
+        <v>428</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>440</v>
-      </c>
-      <c r="N45" t="s" s="2">
-        <v>441</v>
-      </c>
+        <v>430</v>
+      </c>
+      <c r="N45" s="2"/>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>82</v>
@@ -7095,7 +7007,7 @@
         <v>82</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>437</v>
+        <v>426</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>80</v>
@@ -7110,38 +7022,38 @@
         <v>103</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>82</v>
+        <v>432</v>
       </c>
       <c r="AL45" t="s" s="2">
-        <v>442</v>
+        <v>280</v>
       </c>
       <c r="AM45" t="s" s="2">
-        <v>443</v>
+        <v>433</v>
       </c>
       <c r="AN45" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO45" t="s" s="2">
-        <v>82</v>
+        <v>434</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
-        <v>445</v>
+        <v>82</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G46" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H46" t="s" s="2">
         <v>82</v>
@@ -7153,20 +7065,16 @@
         <v>92</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>231</v>
+        <v>442</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>447</v>
-      </c>
-      <c r="N46" t="s" s="2">
-        <v>448</v>
-      </c>
-      <c r="O46" t="s" s="2">
-        <v>449</v>
-      </c>
+        <v>444</v>
+      </c>
+      <c r="N46" s="2"/>
+      <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
         <v>82</v>
       </c>
@@ -7190,11 +7098,13 @@
         <v>82</v>
       </c>
       <c r="X46" t="s" s="2">
-        <v>450</v>
-      </c>
-      <c r="Y46" s="2"/>
+        <v>82</v>
+      </c>
+      <c r="Y46" t="s" s="2">
+        <v>82</v>
+      </c>
       <c r="Z46" t="s" s="2">
-        <v>451</v>
+        <v>82</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>82</v>
@@ -7212,13 +7122,13 @@
         <v>82</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH46" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="AI46" t="s" s="2">
         <v>82</v>
@@ -7230,24 +7140,24 @@
         <v>82</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>442</v>
+        <v>280</v>
       </c>
       <c r="AM46" t="s" s="2">
-        <v>452</v>
+        <v>445</v>
       </c>
       <c r="AN46" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO46" t="s" s="2">
-        <v>453</v>
+        <v>82</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7255,7 +7165,7 @@
       </c>
       <c r="E47" s="2"/>
       <c r="F47" t="s" s="2">
-        <v>455</v>
+        <v>80</v>
       </c>
       <c r="G47" t="s" s="2">
         <v>81</v>
@@ -7270,15 +7180,17 @@
         <v>82</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>456</v>
+        <v>447</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>457</v>
+        <v>448</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>458</v>
-      </c>
-      <c r="N47" s="2"/>
+        <v>449</v>
+      </c>
+      <c r="N47" t="s" s="2">
+        <v>450</v>
+      </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
         <v>82</v>
@@ -7315,17 +7227,19 @@
         <v>82</v>
       </c>
       <c r="AB47" t="s" s="2">
-        <v>459</v>
-      </c>
-      <c r="AC47" s="2"/>
+        <v>82</v>
+      </c>
+      <c r="AC47" t="s" s="2">
+        <v>82</v>
+      </c>
       <c r="AD47" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE47" t="s" s="2">
-        <v>140</v>
+        <v>82</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>80</v>
@@ -7340,484 +7254,18 @@
         <v>103</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>460</v>
+        <v>451</v>
       </c>
       <c r="AL47" t="s" s="2">
-        <v>280</v>
+        <v>134</v>
       </c>
       <c r="AM47" t="s" s="2">
-        <v>461</v>
+        <v>452</v>
       </c>
       <c r="AN47" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO47" t="s" s="2">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="s" s="2">
-        <v>463</v>
-      </c>
-      <c r="B48" t="s" s="2">
-        <v>454</v>
-      </c>
-      <c r="C48" t="s" s="2">
-        <v>464</v>
-      </c>
-      <c r="D48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E48" s="2"/>
-      <c r="F48" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="G48" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K48" t="s" s="2">
-        <v>456</v>
-      </c>
-      <c r="L48" t="s" s="2">
-        <v>465</v>
-      </c>
-      <c r="M48" t="s" s="2">
-        <v>458</v>
-      </c>
-      <c r="N48" s="2"/>
-      <c r="O48" s="2"/>
-      <c r="P48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q48" s="2"/>
-      <c r="R48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF48" t="s" s="2">
-        <v>454</v>
-      </c>
-      <c r="AG48" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH48" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ48" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AK48" t="s" s="2">
-        <v>460</v>
-      </c>
-      <c r="AL48" t="s" s="2">
-        <v>280</v>
-      </c>
-      <c r="AM48" t="s" s="2">
-        <v>461</v>
-      </c>
-      <c r="AN48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO48" t="s" s="2">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="s" s="2">
-        <v>466</v>
-      </c>
-      <c r="B49" t="s" s="2">
-        <v>454</v>
-      </c>
-      <c r="C49" t="s" s="2">
-        <v>467</v>
-      </c>
-      <c r="D49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E49" s="2"/>
-      <c r="F49" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="G49" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K49" t="s" s="2">
-        <v>456</v>
-      </c>
-      <c r="L49" t="s" s="2">
-        <v>468</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>458</v>
-      </c>
-      <c r="N49" s="2"/>
-      <c r="O49" s="2"/>
-      <c r="P49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q49" s="2"/>
-      <c r="R49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF49" t="s" s="2">
-        <v>454</v>
-      </c>
-      <c r="AG49" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH49" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ49" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AK49" t="s" s="2">
-        <v>460</v>
-      </c>
-      <c r="AL49" t="s" s="2">
-        <v>280</v>
-      </c>
-      <c r="AM49" t="s" s="2">
-        <v>461</v>
-      </c>
-      <c r="AN49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO49" t="s" s="2">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="s" s="2">
-        <v>469</v>
-      </c>
-      <c r="B50" t="s" s="2">
-        <v>469</v>
-      </c>
-      <c r="C50" s="2"/>
-      <c r="D50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E50" s="2"/>
-      <c r="F50" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G50" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J50" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K50" t="s" s="2">
-        <v>282</v>
-      </c>
-      <c r="L50" t="s" s="2">
-        <v>470</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>471</v>
-      </c>
-      <c r="N50" s="2"/>
-      <c r="O50" s="2"/>
-      <c r="P50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q50" s="2"/>
-      <c r="R50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF50" t="s" s="2">
-        <v>469</v>
-      </c>
-      <c r="AG50" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH50" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ50" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AK50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL50" t="s" s="2">
-        <v>280</v>
-      </c>
-      <c r="AM50" t="s" s="2">
-        <v>472</v>
-      </c>
-      <c r="AN50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO50" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="s" s="2">
-        <v>473</v>
-      </c>
-      <c r="B51" t="s" s="2">
-        <v>473</v>
-      </c>
-      <c r="C51" s="2"/>
-      <c r="D51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E51" s="2"/>
-      <c r="F51" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G51" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K51" t="s" s="2">
-        <v>474</v>
-      </c>
-      <c r="L51" t="s" s="2">
-        <v>475</v>
-      </c>
-      <c r="M51" t="s" s="2">
-        <v>476</v>
-      </c>
-      <c r="N51" t="s" s="2">
-        <v>477</v>
-      </c>
-      <c r="O51" s="2"/>
-      <c r="P51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q51" s="2"/>
-      <c r="R51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF51" t="s" s="2">
-        <v>473</v>
-      </c>
-      <c r="AG51" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH51" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ51" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AK51" t="s" s="2">
-        <v>478</v>
-      </c>
-      <c r="AL51" t="s" s="2">
-        <v>134</v>
-      </c>
-      <c r="AM51" t="s" s="2">
-        <v>479</v>
-      </c>
-      <c r="AN51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO51" t="s" s="2">
         <v>82</v>
       </c>
     </row>

</xml_diff>